<commit_message>
Update with Index management and Admin modifications
</commit_message>
<xml_diff>
--- a/data/Products.xlsx
+++ b/data/Products.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BA396"/>
+  <dimension ref="A1:BA398"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -58233,9 +58233,316 @@
         <v/>
       </c>
     </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="B397" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="C397" t="str">
+        <v>Drylock</v>
+      </c>
+      <c r="D397" t="str">
+        <v>CZ11</v>
+      </c>
+      <c r="E397" t="str">
+        <v>CZ</v>
+      </c>
+      <c r="F397" t="str">
+        <v>hygiene</v>
+      </c>
+      <c r="G397" t="str">
+        <v>BS</v>
+      </c>
+      <c r="H397" t="str">
+        <v>S</v>
+      </c>
+      <c r="I397" t="str">
+        <v>bico</v>
+      </c>
+      <c r="J397" t="str">
+        <v>G01 - Ovál</v>
+      </c>
+      <c r="K397">
+        <v>12</v>
+      </c>
+      <c r="L397">
+        <v>0</v>
+      </c>
+      <c r="M397" t="str">
+        <v>no treatment</v>
+      </c>
+      <c r="N397" t="str">
+        <v>0 - natur</v>
+      </c>
+      <c r="O397" t="str">
+        <v>Svobodova</v>
+      </c>
+      <c r="P397">
+        <v>0.8473076923076923</v>
+      </c>
+      <c r="Q397">
+        <v>1169.28</v>
+      </c>
+      <c r="R397">
+        <v>1.0093466117383345</v>
+      </c>
+      <c r="S397">
+        <v>0</v>
+      </c>
+      <c r="T397">
+        <v>0.02</v>
+      </c>
+      <c r="U397">
+        <v>0.7</v>
+      </c>
+      <c r="V397">
+        <v>0.6799999999999999</v>
+      </c>
+      <c r="W397">
+        <v>0</v>
+      </c>
+      <c r="X397">
+        <v>0</v>
+      </c>
+      <c r="Y397">
+        <v>0</v>
+      </c>
+      <c r="Z397">
+        <v>0</v>
+      </c>
+      <c r="AA397">
+        <v>0.3</v>
+      </c>
+      <c r="AB397">
+        <v>0</v>
+      </c>
+      <c r="AC397">
+        <v>0</v>
+      </c>
+      <c r="AD397">
+        <v>0</v>
+      </c>
+      <c r="AE397">
+        <v>0</v>
+      </c>
+      <c r="AF397">
+        <v>0</v>
+      </c>
+      <c r="AG397">
+        <v>0</v>
+      </c>
+      <c r="AH397">
+        <v>0</v>
+      </c>
+      <c r="AI397">
+        <v>0</v>
+      </c>
+      <c r="AJ397">
+        <v>0</v>
+      </c>
+      <c r="AK397">
+        <v>1</v>
+      </c>
+      <c r="AL397" t="str">
+        <v>S: PPSB - Mosten NB 425</v>
+      </c>
+      <c r="AM397" t="str">
+        <v>0</v>
+      </c>
+      <c r="AN397">
+        <v>0</v>
+      </c>
+      <c r="AO397">
+        <v>0</v>
+      </c>
+      <c r="AQ397" t="str">
+        <v>S: PE Liten LS87</v>
+      </c>
+      <c r="AS397">
+        <v>0</v>
+      </c>
+      <c r="AT397">
+        <v>0</v>
+      </c>
+      <c r="AU397">
+        <v>0</v>
+      </c>
+      <c r="AV397">
+        <v>0</v>
+      </c>
+      <c r="AW397">
+        <v>0</v>
+      </c>
+      <c r="AX397">
+        <v>0</v>
+      </c>
+      <c r="AY397">
+        <v>0</v>
+      </c>
+      <c r="AZ397">
+        <v>0</v>
+      </c>
+      <c r="BA397">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="B398" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="C398" t="str">
+        <v>Drylock</v>
+      </c>
+      <c r="D398" t="str">
+        <v>CZ11</v>
+      </c>
+      <c r="E398" t="str">
+        <v>CZ</v>
+      </c>
+      <c r="F398" t="str">
+        <v>hygiene</v>
+      </c>
+      <c r="G398" t="str">
+        <v>TS</v>
+      </c>
+      <c r="H398" t="str">
+        <v>S</v>
+      </c>
+      <c r="I398" t="str">
+        <v>Mono</v>
+      </c>
+      <c r="J398" t="str">
+        <v>G08 - honeycombs</v>
+      </c>
+      <c r="K398">
+        <v>12</v>
+      </c>
+      <c r="L398">
+        <v>0</v>
+      </c>
+      <c r="M398" t="str">
+        <v>hydrophilic+Aloe+vitE</v>
+      </c>
+      <c r="N398" t="str">
+        <v>100 - white</v>
+      </c>
+      <c r="O398" t="str">
+        <v>Svobodova</v>
+      </c>
+      <c r="P398">
+        <v>0.8423076923076923</v>
+      </c>
+      <c r="Q398">
+        <v>1169.28</v>
+      </c>
+      <c r="R398">
+        <v>1.0153381669678316</v>
+      </c>
+      <c r="S398">
+        <v>0.08</v>
+      </c>
+      <c r="T398">
+        <v>0.05</v>
+      </c>
+      <c r="U398">
+        <v>0.996</v>
+      </c>
+      <c r="V398">
+        <v>0.866</v>
+      </c>
+      <c r="W398">
+        <v>0</v>
+      </c>
+      <c r="X398">
+        <v>0</v>
+      </c>
+      <c r="Y398">
+        <v>0</v>
+      </c>
+      <c r="Z398">
+        <v>0</v>
+      </c>
+      <c r="AA398">
+        <v>0</v>
+      </c>
+      <c r="AB398">
+        <v>0</v>
+      </c>
+      <c r="AC398">
+        <v>0.005208333333333334</v>
+      </c>
+      <c r="AD398">
+        <v>0.00005</v>
+      </c>
+      <c r="AE398">
+        <v>0.0001</v>
+      </c>
+      <c r="AF398">
+        <v>0.004</v>
+      </c>
+      <c r="AG398">
+        <v>0</v>
+      </c>
+      <c r="AH398">
+        <v>0</v>
+      </c>
+      <c r="AI398">
+        <v>0</v>
+      </c>
+      <c r="AJ398">
+        <v>0</v>
+      </c>
+      <c r="AK398">
+        <v>1.0053583333333336</v>
+      </c>
+      <c r="AL398" t="str">
+        <v>S: PPSB - Mosten NB 425</v>
+      </c>
+      <c r="AM398">
+        <v>0</v>
+      </c>
+      <c r="AN398">
+        <v>0</v>
+      </c>
+      <c r="AO398">
+        <v>0</v>
+      </c>
+      <c r="AS398" t="str">
+        <v>S: Zušl. - Silastol PHP 207</v>
+      </c>
+      <c r="AT398" t="str">
+        <v>Aloe Vera - powder 200x</v>
+      </c>
+      <c r="AU398" t="str">
+        <v>Silastol Care T- Vitamine E</v>
+      </c>
+      <c r="AV398" t="str">
+        <v>S: Pig.  - CC10084467BG bílá 60%</v>
+      </c>
+      <c r="AW398">
+        <v>0</v>
+      </c>
+      <c r="AX398">
+        <v>0</v>
+      </c>
+      <c r="AY398">
+        <v>0</v>
+      </c>
+      <c r="AZ398">
+        <v>0</v>
+      </c>
+      <c r="BA398">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BA396"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BA398"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>